<commit_message>
V02 de ACTIVOS Y RIESGOS
</commit_message>
<xml_diff>
--- a/01_PRIMER_PARCIAL/01_DOCUMENTACION/02_REQUISITOS/01_REQUISITOS_FUNCIONALES_V01.xlsx
+++ b/01_PRIMER_PARCIAL/01_DOCUMENTACION/02_REQUISITOS/01_REQUISITOS_FUNCIONALES_V01.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josecito/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josecito/Desktop/ESPE/SEPTIMO/SOFTWARE SEGURO/36902-DESARROLLO_SOFTWARE_SEGURO-PROYECTOS/01_PRIMER_PARCIAL/01_DOCUMENTACION/02_REQUISITOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D175C944-9D8C-6249-93C9-D57BE94EA4E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{617F9CB3-F56D-F546-9586-80617C6F2E09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="16480" xr2:uid="{401C71C4-BAB8-A749-A636-1C285FBB789A}"/>
+    <workbookView xWindow="15120" yWindow="680" windowWidth="15140" windowHeight="16640" xr2:uid="{401C71C4-BAB8-A749-A636-1C285FBB789A}"/>
   </bookViews>
   <sheets>
     <sheet name="REQUISITOS FUNCIONALES" sheetId="1" r:id="rId1"/>
@@ -698,7 +698,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>25</v>
       </c>

</xml_diff>